<commit_message>
Control de cambios pre finalizada
</commit_message>
<xml_diff>
--- a/EquiposUnidos/app/src/main/res/raw/template_preven_carga.xlsx
+++ b/EquiposUnidos/app/src/main/res/raw/template_preven_carga.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Developer user\android\williApp\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elksi\Android\williApp\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F8FBB6-8DCA-4EFE-BE26-9D34E0089CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3CC28E1-D0B4-4B90-A230-BAE8761A5392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12504" tabRatio="840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FT-MANT-02" sheetId="15" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'FT-MANT-02'!$A$1:$J$109</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'FT-MANT-02'!$A$1:$J$111</definedName>
     <definedName name="DEPENDIENTE2">[1]Hoja1!$C$1:$C$65536</definedName>
     <definedName name="INDEPENDIENTE2">[1]Hoja1!$B$1:$B$65536</definedName>
     <definedName name="INICIO2">[1]Hoja1!$B$1</definedName>
@@ -399,7 +399,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_-[$€-2]* #,##0.00_-;\-[$€-2]* #,##0.00_-;_-[$€-2]* &quot;-&quot;??_-"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -586,6 +586,11 @@
     <font>
       <b/>
       <sz val="16"/>
+      <name val="Muller Regular"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Muller Regular"/>
     </font>
   </fonts>
@@ -1168,7 +1173,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -1271,6 +1276,24 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1280,33 +1303,6 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -1346,6 +1342,12 @@
     <xf numFmtId="0" fontId="24" fillId="25" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1373,13 +1375,7 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1493,20 +1489,44 @@
     <xf numFmtId="0" fontId="24" fillId="25" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="60">
@@ -2349,29 +2369,29 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:J118"/>
+  <dimension ref="B1:J120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="6.88671875" style="18" customWidth="1"/>
-    <col min="2" max="2" width="39.5546875" style="18" customWidth="1"/>
+    <col min="2" max="2" width="56.5546875" style="18" customWidth="1"/>
     <col min="3" max="3" width="63.33203125" style="18" customWidth="1"/>
     <col min="4" max="7" width="13" style="18" customWidth="1"/>
-    <col min="8" max="8" width="23.6640625" style="18" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" style="18" customWidth="1"/>
     <col min="9" max="9" width="31.33203125" style="18" customWidth="1"/>
     <col min="10" max="10" width="29.44140625" style="18" customWidth="1"/>
     <col min="11" max="16384" width="11.44140625" style="18"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:10" s="3" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B1" s="71"/>
-      <c r="C1" s="81" t="s">
+      <c r="B1" s="68"/>
+      <c r="C1" s="78" t="s">
         <v>116</v>
       </c>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="83"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="80"/>
       <c r="I1" s="1" t="s">
         <v>34</v>
       </c>
@@ -2380,13 +2400,13 @@
       </c>
     </row>
     <row r="2" spans="2:10" s="3" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B2" s="72"/>
-      <c r="C2" s="84"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="86"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="83"/>
       <c r="I2" s="4" t="s">
         <v>32</v>
       </c>
@@ -2395,13 +2415,13 @@
       </c>
     </row>
     <row r="3" spans="2:10" s="3" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B3" s="73"/>
-      <c r="C3" s="87"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="89"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="85"/>
+      <c r="E3" s="85"/>
+      <c r="F3" s="85"/>
+      <c r="G3" s="85"/>
+      <c r="H3" s="86"/>
       <c r="I3" s="6" t="s">
         <v>33</v>
       </c>
@@ -2410,30 +2430,30 @@
       </c>
     </row>
     <row r="4" spans="2:10" s="3" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B4" s="74"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="75"/>
-      <c r="H4" s="75"/>
-      <c r="I4" s="75"/>
-      <c r="J4" s="76"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="2:10" s="3" customFormat="1" ht="33" customHeight="1">
       <c r="B5" s="8" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="9"/>
-      <c r="D5" s="96" t="s">
+      <c r="D5" s="93" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="96"/>
-      <c r="F5" s="96"/>
-      <c r="G5" s="96"/>
-      <c r="H5" s="90"/>
-      <c r="I5" s="91"/>
-      <c r="J5" s="77" t="s">
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="87"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="74" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2442,81 +2462,81 @@
         <v>5</v>
       </c>
       <c r="C6" s="9"/>
-      <c r="D6" s="96" t="s">
+      <c r="D6" s="93" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="96"/>
-      <c r="F6" s="96"/>
-      <c r="G6" s="96"/>
-      <c r="H6" s="90"/>
-      <c r="I6" s="91"/>
-      <c r="J6" s="77"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="87"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="74"/>
     </row>
     <row r="7" spans="2:10" s="3" customFormat="1" ht="33" customHeight="1">
       <c r="B7" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="9"/>
-      <c r="D7" s="96" t="s">
+      <c r="D7" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="96"/>
-      <c r="F7" s="96"/>
-      <c r="G7" s="96"/>
-      <c r="H7" s="90"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="98"/>
+      <c r="E7" s="93"/>
+      <c r="F7" s="93"/>
+      <c r="G7" s="93"/>
+      <c r="H7" s="87"/>
+      <c r="I7" s="88"/>
+      <c r="J7" s="95"/>
     </row>
     <row r="8" spans="2:10" s="3" customFormat="1" ht="33" customHeight="1">
       <c r="B8" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="9"/>
-      <c r="D8" s="96" t="s">
+      <c r="D8" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="96"/>
-      <c r="F8" s="96"/>
-      <c r="G8" s="96"/>
-      <c r="H8" s="92" t="s">
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="89" t="s">
         <v>118</v>
       </c>
-      <c r="I8" s="93"/>
-      <c r="J8" s="99"/>
+      <c r="I8" s="90"/>
+      <c r="J8" s="96"/>
     </row>
     <row r="9" spans="2:10" s="3" customFormat="1" ht="42" customHeight="1">
       <c r="B9" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="11"/>
-      <c r="D9" s="97" t="s">
+      <c r="D9" s="94" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="97"/>
-      <c r="F9" s="97"/>
-      <c r="G9" s="97"/>
-      <c r="H9" s="94"/>
-      <c r="I9" s="95"/>
-      <c r="J9" s="100"/>
+      <c r="E9" s="94"/>
+      <c r="F9" s="94"/>
+      <c r="G9" s="94"/>
+      <c r="H9" s="91"/>
+      <c r="I9" s="92"/>
+      <c r="J9" s="97"/>
     </row>
     <row r="10" spans="2:10" s="3" customFormat="1" ht="33" customHeight="1">
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="57"/>
-      <c r="D10" s="58"/>
-      <c r="E10" s="58"/>
-      <c r="F10" s="58"/>
-      <c r="G10" s="58"/>
-      <c r="H10" s="58"/>
-      <c r="I10" s="58"/>
-      <c r="J10" s="57"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="55"/>
+      <c r="E10" s="55"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="55"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="55"/>
+      <c r="J10" s="54"/>
     </row>
     <row r="11" spans="2:10" s="3" customFormat="1" ht="33" customHeight="1">
-      <c r="B11" s="101" t="s">
+      <c r="B11" s="98" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="102"/>
+      <c r="C11" s="99"/>
       <c r="D11" s="20" t="s">
         <v>10</v>
       </c>
@@ -2532,49 +2552,49 @@
       <c r="H11" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="57" t="s">
+      <c r="I11" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="J11" s="57"/>
+      <c r="J11" s="54"/>
     </row>
     <row r="12" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B12" s="48" t="s">
+      <c r="B12" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="46"/>
+      <c r="C12" s="43"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="79"/>
+      <c r="I12" s="75"/>
+      <c r="J12" s="76"/>
     </row>
     <row r="13" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B13" s="80" t="s">
+      <c r="B13" s="77" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="80"/>
+      <c r="C13" s="77"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
-      <c r="I13" s="36"/>
-      <c r="J13" s="35"/>
+      <c r="I13" s="42"/>
+      <c r="J13" s="41"/>
     </row>
     <row r="14" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="47"/>
+      <c r="C14" s="44"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="35"/>
+      <c r="I14" s="42"/>
+      <c r="J14" s="41"/>
     </row>
     <row r="15" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B15" s="23" t="s">
@@ -2590,30 +2610,30 @@
       <c r="J15" s="22"/>
     </row>
     <row r="16" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B16" s="55" t="s">
+      <c r="B16" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="56"/>
+      <c r="C16" s="53"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
-      <c r="I16" s="36"/>
-      <c r="J16" s="35"/>
+      <c r="I16" s="42"/>
+      <c r="J16" s="41"/>
     </row>
     <row r="17" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="52" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="56"/>
+      <c r="C17" s="53"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
       <c r="H17" s="9"/>
-      <c r="I17" s="36"/>
-      <c r="J17" s="35"/>
+      <c r="I17" s="42"/>
+      <c r="J17" s="41"/>
     </row>
     <row r="18" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B18" s="16" t="s">
@@ -2625,164 +2645,164 @@
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
       <c r="H18" s="9"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="35"/>
+      <c r="I18" s="42"/>
+      <c r="J18" s="41"/>
     </row>
     <row r="19" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B19" s="55" t="s">
+      <c r="B19" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="56"/>
+      <c r="C19" s="53"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
       <c r="H19" s="9"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="35"/>
+      <c r="I19" s="42"/>
+      <c r="J19" s="41"/>
     </row>
     <row r="20" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B20" s="55" t="s">
+      <c r="B20" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="56"/>
+      <c r="C20" s="53"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
       <c r="H20" s="9"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="35"/>
+      <c r="I20" s="42"/>
+      <c r="J20" s="41"/>
     </row>
     <row r="21" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B21" s="55" t="s">
+      <c r="B21" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="56"/>
+      <c r="C21" s="53"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
       <c r="H21" s="9"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="35"/>
+      <c r="I21" s="42"/>
+      <c r="J21" s="41"/>
     </row>
     <row r="22" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B22" s="55" t="s">
+      <c r="B22" s="52" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="56"/>
+      <c r="C22" s="53"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
-      <c r="I22" s="36"/>
-      <c r="J22" s="35"/>
+      <c r="I22" s="42"/>
+      <c r="J22" s="41"/>
     </row>
     <row r="23" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B23" s="48" t="s">
+      <c r="B23" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="C23" s="47"/>
+      <c r="C23" s="44"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
-      <c r="I23" s="36"/>
-      <c r="J23" s="35"/>
+      <c r="I23" s="42"/>
+      <c r="J23" s="41"/>
     </row>
     <row r="24" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B24" s="48" t="s">
+      <c r="B24" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="47"/>
+      <c r="C24" s="44"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
       <c r="H24" s="9"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="35"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="41"/>
     </row>
     <row r="25" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B25" s="55" t="s">
+      <c r="B25" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="56"/>
+      <c r="C25" s="53"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
-      <c r="I25" s="36"/>
-      <c r="J25" s="35"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="41"/>
     </row>
     <row r="26" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B26" s="55" t="s">
+      <c r="B26" s="52" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="56"/>
+      <c r="C26" s="53"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
-      <c r="I26" s="36"/>
-      <c r="J26" s="35"/>
+      <c r="I26" s="42"/>
+      <c r="J26" s="41"/>
     </row>
     <row r="27" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B27" s="48" t="s">
+      <c r="B27" s="45" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="47"/>
+      <c r="C27" s="44"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
       <c r="H27" s="9"/>
-      <c r="I27" s="36"/>
-      <c r="J27" s="35"/>
+      <c r="I27" s="42"/>
+      <c r="J27" s="41"/>
     </row>
     <row r="28" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B28" s="55" t="s">
+      <c r="B28" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="C28" s="56"/>
+      <c r="C28" s="53"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
       <c r="H28" s="9"/>
-      <c r="I28" s="36"/>
-      <c r="J28" s="35"/>
+      <c r="I28" s="42"/>
+      <c r="J28" s="41"/>
     </row>
     <row r="29" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B29" s="55" t="s">
+      <c r="B29" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="56"/>
+      <c r="C29" s="53"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
       <c r="H29" s="9"/>
-      <c r="I29" s="36"/>
-      <c r="J29" s="35"/>
+      <c r="I29" s="42"/>
+      <c r="J29" s="41"/>
     </row>
     <row r="30" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B30" s="68" t="s">
+      <c r="B30" s="56" t="s">
         <v>112</v>
       </c>
-      <c r="C30" s="69"/>
+      <c r="C30" s="67"/>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
       <c r="H30" s="9"/>
-      <c r="I30" s="36"/>
-      <c r="J30" s="35"/>
+      <c r="I30" s="42"/>
+      <c r="J30" s="41"/>
     </row>
     <row r="31" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B31" s="23" t="s">
@@ -2798,43 +2818,43 @@
       <c r="J31" s="22"/>
     </row>
     <row r="32" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B32" s="55" t="s">
+      <c r="B32" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="C32" s="56"/>
+      <c r="C32" s="53"/>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
-      <c r="I32" s="36"/>
-      <c r="J32" s="35"/>
+      <c r="I32" s="42"/>
+      <c r="J32" s="41"/>
     </row>
     <row r="33" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B33" s="55" t="s">
+      <c r="B33" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="C33" s="56"/>
+      <c r="C33" s="53"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
-      <c r="I33" s="36"/>
-      <c r="J33" s="35"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="41"/>
     </row>
     <row r="34" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B34" s="55" t="s">
+      <c r="B34" s="52" t="s">
         <v>49</v>
       </c>
-      <c r="C34" s="56"/>
+      <c r="C34" s="53"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
       <c r="H34" s="9"/>
-      <c r="I34" s="36"/>
-      <c r="J34" s="35"/>
+      <c r="I34" s="42"/>
+      <c r="J34" s="41"/>
     </row>
     <row r="35" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B35" s="23" t="s">
@@ -2850,43 +2870,43 @@
       <c r="J35" s="22"/>
     </row>
     <row r="36" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B36" s="55" t="s">
+      <c r="B36" s="52" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="56"/>
+      <c r="C36" s="53"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
       <c r="H36" s="9"/>
-      <c r="I36" s="36"/>
-      <c r="J36" s="35"/>
+      <c r="I36" s="42"/>
+      <c r="J36" s="41"/>
     </row>
     <row r="37" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B37" s="55" t="s">
+      <c r="B37" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="56"/>
+      <c r="C37" s="53"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
       <c r="H37" s="9"/>
-      <c r="I37" s="36"/>
-      <c r="J37" s="35"/>
+      <c r="I37" s="42"/>
+      <c r="J37" s="41"/>
     </row>
     <row r="38" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B38" s="55" t="s">
+      <c r="B38" s="52" t="s">
         <v>61</v>
       </c>
-      <c r="C38" s="56"/>
+      <c r="C38" s="53"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
       <c r="H38" s="9"/>
-      <c r="I38" s="36"/>
-      <c r="J38" s="35"/>
+      <c r="I38" s="42"/>
+      <c r="J38" s="41"/>
     </row>
     <row r="39" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B39" s="23" t="s">
@@ -2902,43 +2922,43 @@
       <c r="J39" s="22"/>
     </row>
     <row r="40" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B40" s="55" t="s">
+      <c r="B40" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="C40" s="56"/>
+      <c r="C40" s="53"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
       <c r="H40" s="9"/>
-      <c r="I40" s="36"/>
-      <c r="J40" s="35"/>
+      <c r="I40" s="42"/>
+      <c r="J40" s="41"/>
     </row>
     <row r="41" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B41" s="55" t="s">
+      <c r="B41" s="52" t="s">
         <v>103</v>
       </c>
-      <c r="C41" s="56"/>
+      <c r="C41" s="53"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
       <c r="F41" s="9"/>
       <c r="G41" s="9"/>
       <c r="H41" s="9"/>
-      <c r="I41" s="36"/>
-      <c r="J41" s="35"/>
+      <c r="I41" s="42"/>
+      <c r="J41" s="41"/>
     </row>
     <row r="42" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B42" s="55" t="s">
+      <c r="B42" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="C42" s="56"/>
+      <c r="C42" s="53"/>
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
       <c r="H42" s="9"/>
-      <c r="I42" s="36"/>
-      <c r="J42" s="35"/>
+      <c r="I42" s="42"/>
+      <c r="J42" s="41"/>
     </row>
     <row r="43" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B43" s="16" t="s">
@@ -2950,8 +2970,8 @@
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
       <c r="H43" s="9"/>
-      <c r="I43" s="36"/>
-      <c r="J43" s="35"/>
+      <c r="I43" s="42"/>
+      <c r="J43" s="41"/>
     </row>
     <row r="44" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B44" s="16" t="s">
@@ -2963,229 +2983,229 @@
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
       <c r="H44" s="9"/>
-      <c r="I44" s="36"/>
-      <c r="J44" s="35"/>
+      <c r="I44" s="42"/>
+      <c r="J44" s="41"/>
     </row>
     <row r="45" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B45" s="48" t="s">
+      <c r="B45" s="45" t="s">
         <v>114</v>
       </c>
-      <c r="C45" s="46"/>
+      <c r="C45" s="43"/>
       <c r="D45" s="9"/>
       <c r="E45" s="9"/>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
       <c r="H45" s="9"/>
-      <c r="I45" s="36"/>
-      <c r="J45" s="35"/>
+      <c r="I45" s="42"/>
+      <c r="J45" s="41"/>
     </row>
     <row r="46" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B46" s="105" t="s">
+      <c r="B46" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="C46" s="103"/>
-      <c r="D46" s="104"/>
-      <c r="E46" s="104"/>
-      <c r="F46" s="104"/>
-      <c r="G46" s="104"/>
-      <c r="H46" s="104"/>
-      <c r="I46" s="103"/>
-      <c r="J46" s="103"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="35"/>
+      <c r="E46" s="35"/>
+      <c r="F46" s="35"/>
+      <c r="G46" s="35"/>
+      <c r="H46" s="35"/>
+      <c r="I46" s="34"/>
+      <c r="J46" s="34"/>
     </row>
     <row r="47" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B47" s="68" t="s">
+      <c r="B47" s="56" t="s">
         <v>105</v>
       </c>
-      <c r="C47" s="69"/>
+      <c r="C47" s="67"/>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
       <c r="H47" s="9"/>
-      <c r="I47" s="34"/>
-      <c r="J47" s="35"/>
+      <c r="I47" s="40"/>
+      <c r="J47" s="41"/>
     </row>
     <row r="48" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B48" s="48" t="s">
+      <c r="B48" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="47"/>
+      <c r="C48" s="44"/>
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
       <c r="H48" s="9"/>
-      <c r="I48" s="36"/>
-      <c r="J48" s="35"/>
+      <c r="I48" s="42"/>
+      <c r="J48" s="41"/>
     </row>
     <row r="49" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B49" s="48" t="s">
+      <c r="B49" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="C49" s="47"/>
+      <c r="C49" s="44"/>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
       <c r="H49" s="9"/>
-      <c r="I49" s="36"/>
-      <c r="J49" s="35"/>
+      <c r="I49" s="42"/>
+      <c r="J49" s="41"/>
     </row>
     <row r="50" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B50" s="48" t="s">
+      <c r="B50" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="C50" s="47"/>
+      <c r="C50" s="44"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
-      <c r="I50" s="36"/>
-      <c r="J50" s="35"/>
+      <c r="I50" s="42"/>
+      <c r="J50" s="41"/>
     </row>
     <row r="51" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B51" s="48" t="s">
+      <c r="B51" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="C51" s="47"/>
+      <c r="C51" s="44"/>
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
       <c r="F51" s="9"/>
       <c r="G51" s="9"/>
       <c r="H51" s="9"/>
-      <c r="I51" s="36"/>
-      <c r="J51" s="35"/>
+      <c r="I51" s="42"/>
+      <c r="J51" s="41"/>
     </row>
     <row r="52" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B52" s="105" t="s">
+      <c r="B52" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C52" s="103"/>
-      <c r="D52" s="104"/>
-      <c r="E52" s="104"/>
-      <c r="F52" s="104"/>
-      <c r="G52" s="104"/>
-      <c r="H52" s="104"/>
+      <c r="C52" s="34"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="35"/>
+      <c r="F52" s="35"/>
+      <c r="G52" s="35"/>
+      <c r="H52" s="35"/>
       <c r="I52" s="21"/>
       <c r="J52" s="22"/>
     </row>
     <row r="53" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B53" s="48" t="s">
+      <c r="B53" s="45" t="s">
         <v>63</v>
       </c>
-      <c r="C53" s="47"/>
+      <c r="C53" s="44"/>
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
       <c r="H53" s="9"/>
-      <c r="I53" s="36"/>
-      <c r="J53" s="35"/>
+      <c r="I53" s="42"/>
+      <c r="J53" s="41"/>
     </row>
     <row r="54" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B54" s="48" t="s">
+      <c r="B54" s="45" t="s">
         <v>113</v>
       </c>
-      <c r="C54" s="47"/>
+      <c r="C54" s="44"/>
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
       <c r="H54" s="9"/>
-      <c r="I54" s="36"/>
-      <c r="J54" s="35"/>
+      <c r="I54" s="42"/>
+      <c r="J54" s="41"/>
     </row>
     <row r="55" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B55" s="48" t="s">
+      <c r="B55" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="C55" s="47"/>
+      <c r="C55" s="44"/>
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
       <c r="H55" s="9"/>
-      <c r="I55" s="36"/>
-      <c r="J55" s="35"/>
+      <c r="I55" s="42"/>
+      <c r="J55" s="41"/>
     </row>
     <row r="56" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B56" s="48" t="s">
+      <c r="B56" s="45" t="s">
         <v>65</v>
       </c>
-      <c r="C56" s="47"/>
+      <c r="C56" s="44"/>
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
       <c r="F56" s="9"/>
       <c r="G56" s="9"/>
       <c r="H56" s="9"/>
-      <c r="I56" s="36"/>
-      <c r="J56" s="35"/>
+      <c r="I56" s="42"/>
+      <c r="J56" s="41"/>
     </row>
     <row r="57" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B57" s="48" t="s">
+      <c r="B57" s="45" t="s">
         <v>107</v>
       </c>
-      <c r="C57" s="47"/>
+      <c r="C57" s="44"/>
       <c r="D57" s="9"/>
       <c r="E57" s="9"/>
       <c r="F57" s="9"/>
       <c r="G57" s="9"/>
       <c r="H57" s="9"/>
-      <c r="I57" s="36"/>
-      <c r="J57" s="35"/>
+      <c r="I57" s="42"/>
+      <c r="J57" s="41"/>
     </row>
     <row r="58" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B58" s="48" t="s">
+      <c r="B58" s="45" t="s">
         <v>108</v>
       </c>
-      <c r="C58" s="47"/>
+      <c r="C58" s="44"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
       <c r="H58" s="9"/>
-      <c r="I58" s="36"/>
-      <c r="J58" s="35"/>
+      <c r="I58" s="42"/>
+      <c r="J58" s="41"/>
     </row>
     <row r="59" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B59" s="48" t="s">
+      <c r="B59" s="45" t="s">
         <v>66</v>
       </c>
-      <c r="C59" s="47"/>
+      <c r="C59" s="44"/>
       <c r="D59" s="9"/>
       <c r="E59" s="9"/>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
       <c r="H59" s="9"/>
-      <c r="I59" s="36"/>
-      <c r="J59" s="35"/>
+      <c r="I59" s="42"/>
+      <c r="J59" s="41"/>
     </row>
     <row r="60" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B60" s="48" t="s">
+      <c r="B60" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="C60" s="47"/>
+      <c r="C60" s="44"/>
       <c r="D60" s="9"/>
       <c r="E60" s="9"/>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
       <c r="H60" s="9"/>
-      <c r="I60" s="36"/>
-      <c r="J60" s="35"/>
+      <c r="I60" s="42"/>
+      <c r="J60" s="41"/>
     </row>
     <row r="61" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B61" s="48" t="s">
+      <c r="B61" s="45" t="s">
         <v>74</v>
       </c>
-      <c r="C61" s="47"/>
+      <c r="C61" s="44"/>
       <c r="D61" s="9"/>
       <c r="E61" s="9"/>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
       <c r="H61" s="9"/>
-      <c r="I61" s="36"/>
-      <c r="J61" s="35"/>
+      <c r="I61" s="42"/>
+      <c r="J61" s="41"/>
     </row>
     <row r="62" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B62" s="23" t="s">
@@ -3201,56 +3221,56 @@
       <c r="J62" s="22"/>
     </row>
     <row r="63" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B63" s="48" t="s">
+      <c r="B63" s="45" t="s">
         <v>71</v>
       </c>
-      <c r="C63" s="47"/>
+      <c r="C63" s="44"/>
       <c r="D63" s="9"/>
       <c r="E63" s="9"/>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
       <c r="H63" s="9"/>
-      <c r="I63" s="36"/>
-      <c r="J63" s="35"/>
+      <c r="I63" s="42"/>
+      <c r="J63" s="41"/>
     </row>
     <row r="64" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B64" s="48" t="s">
+      <c r="B64" s="45" t="s">
         <v>79</v>
       </c>
-      <c r="C64" s="47"/>
+      <c r="C64" s="44"/>
       <c r="D64" s="9"/>
       <c r="E64" s="9"/>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
       <c r="H64" s="9"/>
-      <c r="I64" s="36"/>
-      <c r="J64" s="35"/>
+      <c r="I64" s="42"/>
+      <c r="J64" s="41"/>
     </row>
     <row r="65" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B65" s="48" t="s">
+      <c r="B65" s="45" t="s">
         <v>72</v>
       </c>
-      <c r="C65" s="47"/>
+      <c r="C65" s="44"/>
       <c r="D65" s="9"/>
       <c r="E65" s="9"/>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
       <c r="H65" s="9"/>
-      <c r="I65" s="36"/>
-      <c r="J65" s="35"/>
+      <c r="I65" s="42"/>
+      <c r="J65" s="41"/>
     </row>
     <row r="66" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B66" s="48" t="s">
+      <c r="B66" s="45" t="s">
         <v>69</v>
       </c>
-      <c r="C66" s="47"/>
+      <c r="C66" s="44"/>
       <c r="D66" s="9"/>
       <c r="E66" s="9"/>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
       <c r="H66" s="9"/>
-      <c r="I66" s="36"/>
-      <c r="J66" s="35"/>
+      <c r="I66" s="42"/>
+      <c r="J66" s="41"/>
     </row>
     <row r="67" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B67" s="23" t="s">
@@ -3266,56 +3286,56 @@
       <c r="J67" s="22"/>
     </row>
     <row r="68" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B68" s="48" t="s">
+      <c r="B68" s="45" t="s">
         <v>73</v>
       </c>
-      <c r="C68" s="47"/>
+      <c r="C68" s="44"/>
       <c r="D68" s="9"/>
       <c r="E68" s="9"/>
       <c r="F68" s="9"/>
       <c r="G68" s="9"/>
       <c r="H68" s="9"/>
-      <c r="I68" s="48"/>
-      <c r="J68" s="47"/>
+      <c r="I68" s="45"/>
+      <c r="J68" s="44"/>
     </row>
     <row r="69" spans="2:10" s="3" customFormat="1" ht="21.75" customHeight="1">
-      <c r="B69" s="55" t="s">
+      <c r="B69" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="C69" s="56"/>
+      <c r="C69" s="53"/>
       <c r="D69" s="9"/>
       <c r="E69" s="9"/>
       <c r="F69" s="9"/>
       <c r="G69" s="9"/>
       <c r="H69" s="9"/>
-      <c r="I69" s="36"/>
-      <c r="J69" s="35"/>
+      <c r="I69" s="42"/>
+      <c r="J69" s="41"/>
     </row>
     <row r="70" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B70" s="48" t="s">
+      <c r="B70" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="C70" s="47"/>
+      <c r="C70" s="44"/>
       <c r="D70" s="9"/>
       <c r="E70" s="9"/>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
       <c r="H70" s="9"/>
-      <c r="I70" s="36"/>
-      <c r="J70" s="35"/>
+      <c r="I70" s="42"/>
+      <c r="J70" s="41"/>
     </row>
     <row r="71" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B71" s="48" t="s">
+      <c r="B71" s="45" t="s">
         <v>76</v>
       </c>
-      <c r="C71" s="47"/>
+      <c r="C71" s="44"/>
       <c r="D71" s="9"/>
       <c r="E71" s="9"/>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
       <c r="H71" s="9"/>
-      <c r="I71" s="36"/>
-      <c r="J71" s="35"/>
+      <c r="I71" s="42"/>
+      <c r="J71" s="41"/>
     </row>
     <row r="72" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B72" s="23" t="s">
@@ -3331,30 +3351,30 @@
       <c r="J72" s="22"/>
     </row>
     <row r="73" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B73" s="65" t="s">
+      <c r="B73" s="64" t="s">
         <v>77</v>
       </c>
-      <c r="C73" s="66"/>
+      <c r="C73" s="65"/>
       <c r="D73" s="9"/>
       <c r="E73" s="9"/>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
       <c r="H73" s="9"/>
-      <c r="I73" s="36"/>
-      <c r="J73" s="35"/>
+      <c r="I73" s="42"/>
+      <c r="J73" s="41"/>
     </row>
     <row r="74" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B74" s="65" t="s">
+      <c r="B74" s="64" t="s">
         <v>78</v>
       </c>
-      <c r="C74" s="67"/>
+      <c r="C74" s="66"/>
       <c r="D74" s="9"/>
       <c r="E74" s="9"/>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
       <c r="H74" s="9"/>
-      <c r="I74" s="46"/>
-      <c r="J74" s="47"/>
+      <c r="I74" s="43"/>
+      <c r="J74" s="44"/>
     </row>
     <row r="75" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B75" s="23" t="s">
@@ -3379,21 +3399,21 @@
       <c r="F76" s="9"/>
       <c r="G76" s="9"/>
       <c r="H76" s="9"/>
-      <c r="I76" s="36"/>
-      <c r="J76" s="35"/>
+      <c r="I76" s="42"/>
+      <c r="J76" s="41"/>
     </row>
     <row r="77" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B77" s="48" t="s">
+      <c r="B77" s="45" t="s">
         <v>81</v>
       </c>
-      <c r="C77" s="47"/>
+      <c r="C77" s="44"/>
       <c r="D77" s="9"/>
       <c r="E77" s="9"/>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
       <c r="H77" s="9"/>
-      <c r="I77" s="36"/>
-      <c r="J77" s="35"/>
+      <c r="I77" s="42"/>
+      <c r="J77" s="41"/>
     </row>
     <row r="78" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B78" s="23" t="s">
@@ -3409,30 +3429,30 @@
       <c r="J78" s="22"/>
     </row>
     <row r="79" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B79" s="48" t="s">
+      <c r="B79" s="45" t="s">
         <v>109</v>
       </c>
-      <c r="C79" s="47"/>
+      <c r="C79" s="44"/>
       <c r="D79" s="9"/>
       <c r="E79" s="9"/>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
       <c r="H79" s="9"/>
-      <c r="I79" s="36"/>
-      <c r="J79" s="35"/>
+      <c r="I79" s="42"/>
+      <c r="J79" s="41"/>
     </row>
     <row r="80" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B80" s="65" t="s">
+      <c r="B80" s="64" t="s">
         <v>83</v>
       </c>
-      <c r="C80" s="66"/>
+      <c r="C80" s="65"/>
       <c r="D80" s="9"/>
       <c r="E80" s="9"/>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
       <c r="H80" s="9"/>
-      <c r="I80" s="36"/>
-      <c r="J80" s="35"/>
+      <c r="I80" s="42"/>
+      <c r="J80" s="41"/>
     </row>
     <row r="81" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B81" s="12" t="s">
@@ -3444,408 +3464,408 @@
       <c r="F81" s="9"/>
       <c r="G81" s="9"/>
       <c r="H81" s="9"/>
-      <c r="I81" s="36"/>
-      <c r="J81" s="35"/>
+      <c r="I81" s="42"/>
+      <c r="J81" s="41"/>
     </row>
     <row r="82" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B82" s="68" t="s">
+      <c r="B82" s="56" t="s">
         <v>110</v>
       </c>
-      <c r="C82" s="70"/>
+      <c r="C82" s="57"/>
       <c r="D82" s="9"/>
       <c r="E82" s="9"/>
       <c r="F82" s="9"/>
       <c r="G82" s="9"/>
       <c r="H82" s="9"/>
-      <c r="I82" s="36"/>
-      <c r="J82" s="35"/>
+      <c r="I82" s="42"/>
+      <c r="J82" s="41"/>
     </row>
     <row r="83" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B83" s="48" t="s">
+      <c r="B83" s="45" t="s">
         <v>85</v>
       </c>
-      <c r="C83" s="47"/>
+      <c r="C83" s="44"/>
       <c r="D83" s="9"/>
       <c r="E83" s="9"/>
       <c r="F83" s="9"/>
       <c r="G83" s="9"/>
       <c r="H83" s="9"/>
-      <c r="I83" s="36"/>
-      <c r="J83" s="35"/>
+      <c r="I83" s="42"/>
+      <c r="J83" s="41"/>
     </row>
     <row r="84" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B84" s="48" t="s">
+      <c r="B84" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="C84" s="47"/>
+      <c r="C84" s="44"/>
       <c r="D84" s="9"/>
       <c r="E84" s="9"/>
       <c r="F84" s="9"/>
       <c r="G84" s="9"/>
       <c r="H84" s="9"/>
-      <c r="I84" s="36"/>
-      <c r="J84" s="35"/>
+      <c r="I84" s="42"/>
+      <c r="J84" s="41"/>
     </row>
     <row r="85" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B85" s="48" t="s">
+      <c r="B85" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="C85" s="47"/>
+      <c r="C85" s="44"/>
       <c r="D85" s="9"/>
       <c r="E85" s="9"/>
       <c r="F85" s="9"/>
       <c r="G85" s="9"/>
       <c r="H85" s="9"/>
-      <c r="I85" s="36"/>
-      <c r="J85" s="35"/>
+      <c r="I85" s="42"/>
+      <c r="J85" s="41"/>
     </row>
     <row r="86" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B86" s="48" t="s">
+      <c r="B86" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="C86" s="47"/>
+      <c r="C86" s="44"/>
       <c r="D86" s="9"/>
       <c r="E86" s="9"/>
       <c r="F86" s="9"/>
       <c r="G86" s="9"/>
       <c r="H86" s="9"/>
-      <c r="I86" s="36"/>
-      <c r="J86" s="35"/>
+      <c r="I86" s="42"/>
+      <c r="J86" s="41"/>
     </row>
     <row r="87" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B87" s="107"/>
-      <c r="C87" s="106"/>
-      <c r="D87" s="104"/>
-      <c r="E87" s="104"/>
-      <c r="F87" s="104"/>
-      <c r="G87" s="104"/>
-      <c r="H87" s="104"/>
+      <c r="B87" s="38"/>
+      <c r="C87" s="37"/>
+      <c r="D87" s="35"/>
+      <c r="E87" s="35"/>
+      <c r="F87" s="35"/>
+      <c r="G87" s="35"/>
+      <c r="H87" s="35"/>
       <c r="I87" s="15"/>
       <c r="J87" s="13"/>
     </row>
     <row r="88" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
-      <c r="B88" s="57" t="s">
+      <c r="B88" s="54" t="s">
         <v>88</v>
       </c>
-      <c r="C88" s="58"/>
-      <c r="D88" s="58"/>
-      <c r="E88" s="58"/>
-      <c r="F88" s="58"/>
-      <c r="G88" s="58"/>
-      <c r="H88" s="58"/>
-      <c r="I88" s="58"/>
-      <c r="J88" s="57"/>
+      <c r="C88" s="55"/>
+      <c r="D88" s="55"/>
+      <c r="E88" s="55"/>
+      <c r="F88" s="55"/>
+      <c r="G88" s="55"/>
+      <c r="H88" s="55"/>
+      <c r="I88" s="55"/>
+      <c r="J88" s="54"/>
     </row>
     <row r="89" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B89" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="C89" s="36"/>
-      <c r="D89" s="34"/>
-      <c r="E89" s="35"/>
-      <c r="F89" s="49" t="s">
+      <c r="C89" s="42"/>
+      <c r="D89" s="40"/>
+      <c r="E89" s="41"/>
+      <c r="F89" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G89" s="50"/>
-      <c r="H89" s="51"/>
-      <c r="I89" s="36"/>
-      <c r="J89" s="35"/>
+      <c r="G89" s="47"/>
+      <c r="H89" s="48"/>
+      <c r="I89" s="42"/>
+      <c r="J89" s="41"/>
     </row>
     <row r="90" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B90" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="C90" s="36"/>
-      <c r="D90" s="34"/>
-      <c r="E90" s="35"/>
-      <c r="F90" s="49" t="s">
+      <c r="C90" s="42"/>
+      <c r="D90" s="40"/>
+      <c r="E90" s="41"/>
+      <c r="F90" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G90" s="50"/>
-      <c r="H90" s="51"/>
-      <c r="I90" s="36"/>
-      <c r="J90" s="35"/>
+      <c r="G90" s="47"/>
+      <c r="H90" s="48"/>
+      <c r="I90" s="42"/>
+      <c r="J90" s="41"/>
     </row>
     <row r="91" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B91" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="C91" s="36"/>
-      <c r="D91" s="34"/>
-      <c r="E91" s="35"/>
-      <c r="F91" s="49" t="s">
+      <c r="C91" s="42"/>
+      <c r="D91" s="40"/>
+      <c r="E91" s="41"/>
+      <c r="F91" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G91" s="50"/>
-      <c r="H91" s="51"/>
-      <c r="I91" s="36"/>
-      <c r="J91" s="35"/>
+      <c r="G91" s="47"/>
+      <c r="H91" s="48"/>
+      <c r="I91" s="42"/>
+      <c r="J91" s="41"/>
     </row>
     <row r="92" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B92" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="C92" s="36"/>
-      <c r="D92" s="34"/>
-      <c r="E92" s="35"/>
-      <c r="F92" s="49" t="s">
+      <c r="C92" s="42"/>
+      <c r="D92" s="40"/>
+      <c r="E92" s="41"/>
+      <c r="F92" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G92" s="50"/>
-      <c r="H92" s="51"/>
-      <c r="I92" s="36"/>
-      <c r="J92" s="35"/>
+      <c r="G92" s="47"/>
+      <c r="H92" s="48"/>
+      <c r="I92" s="42"/>
+      <c r="J92" s="41"/>
     </row>
     <row r="93" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B93" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="C93" s="36"/>
-      <c r="D93" s="34"/>
-      <c r="E93" s="35"/>
-      <c r="F93" s="49" t="s">
+      <c r="C93" s="42"/>
+      <c r="D93" s="40"/>
+      <c r="E93" s="41"/>
+      <c r="F93" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G93" s="50"/>
-      <c r="H93" s="51"/>
-      <c r="I93" s="36"/>
-      <c r="J93" s="35"/>
+      <c r="G93" s="47"/>
+      <c r="H93" s="48"/>
+      <c r="I93" s="42"/>
+      <c r="J93" s="41"/>
     </row>
     <row r="94" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B94" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="C94" s="36"/>
-      <c r="D94" s="34"/>
-      <c r="E94" s="35"/>
-      <c r="F94" s="49" t="s">
+      <c r="C94" s="42"/>
+      <c r="D94" s="40"/>
+      <c r="E94" s="41"/>
+      <c r="F94" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G94" s="50"/>
-      <c r="H94" s="51"/>
-      <c r="I94" s="36"/>
-      <c r="J94" s="35"/>
+      <c r="G94" s="47"/>
+      <c r="H94" s="48"/>
+      <c r="I94" s="42"/>
+      <c r="J94" s="41"/>
     </row>
     <row r="95" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B95" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C95" s="36"/>
-      <c r="D95" s="34"/>
-      <c r="E95" s="35"/>
-      <c r="F95" s="49" t="s">
+      <c r="C95" s="42"/>
+      <c r="D95" s="40"/>
+      <c r="E95" s="41"/>
+      <c r="F95" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G95" s="50"/>
-      <c r="H95" s="51"/>
-      <c r="I95" s="36"/>
-      <c r="J95" s="35"/>
+      <c r="G95" s="47"/>
+      <c r="H95" s="48"/>
+      <c r="I95" s="42"/>
+      <c r="J95" s="41"/>
     </row>
     <row r="96" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B96" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="C96" s="36"/>
-      <c r="D96" s="34"/>
-      <c r="E96" s="35"/>
-      <c r="F96" s="49" t="s">
+      <c r="C96" s="42"/>
+      <c r="D96" s="40"/>
+      <c r="E96" s="41"/>
+      <c r="F96" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G96" s="50"/>
-      <c r="H96" s="51"/>
-      <c r="I96" s="36"/>
-      <c r="J96" s="35"/>
+      <c r="G96" s="47"/>
+      <c r="H96" s="48"/>
+      <c r="I96" s="42"/>
+      <c r="J96" s="41"/>
     </row>
     <row r="97" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B97" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="C97" s="36"/>
-      <c r="D97" s="34"/>
-      <c r="E97" s="35"/>
-      <c r="F97" s="49" t="s">
+      <c r="C97" s="42"/>
+      <c r="D97" s="40"/>
+      <c r="E97" s="41"/>
+      <c r="F97" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G97" s="50"/>
-      <c r="H97" s="51"/>
-      <c r="I97" s="36"/>
-      <c r="J97" s="35"/>
+      <c r="G97" s="47"/>
+      <c r="H97" s="48"/>
+      <c r="I97" s="42"/>
+      <c r="J97" s="41"/>
     </row>
     <row r="98" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B98" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="C98" s="36"/>
-      <c r="D98" s="34"/>
-      <c r="E98" s="35"/>
-      <c r="F98" s="49" t="s">
+      <c r="C98" s="42"/>
+      <c r="D98" s="40"/>
+      <c r="E98" s="41"/>
+      <c r="F98" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G98" s="50"/>
-      <c r="H98" s="51"/>
-      <c r="I98" s="36"/>
-      <c r="J98" s="35"/>
+      <c r="G98" s="47"/>
+      <c r="H98" s="48"/>
+      <c r="I98" s="42"/>
+      <c r="J98" s="41"/>
     </row>
     <row r="99" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B99" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="C99" s="36"/>
-      <c r="D99" s="34"/>
-      <c r="E99" s="35"/>
-      <c r="F99" s="49" t="s">
+      <c r="C99" s="42"/>
+      <c r="D99" s="40"/>
+      <c r="E99" s="41"/>
+      <c r="F99" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G99" s="50"/>
-      <c r="H99" s="51"/>
-      <c r="I99" s="36"/>
-      <c r="J99" s="35"/>
+      <c r="G99" s="47"/>
+      <c r="H99" s="48"/>
+      <c r="I99" s="42"/>
+      <c r="J99" s="41"/>
     </row>
     <row r="100" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B100" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="C100" s="36"/>
-      <c r="D100" s="34"/>
-      <c r="E100" s="35"/>
-      <c r="F100" s="49" t="s">
+      <c r="C100" s="42"/>
+      <c r="D100" s="40"/>
+      <c r="E100" s="41"/>
+      <c r="F100" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="G100" s="50"/>
-      <c r="H100" s="51"/>
-      <c r="I100" s="36"/>
-      <c r="J100" s="35"/>
+      <c r="G100" s="47"/>
+      <c r="H100" s="48"/>
+      <c r="I100" s="42"/>
+      <c r="J100" s="41"/>
     </row>
     <row r="101" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B101" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="C101" s="34"/>
-      <c r="D101" s="34"/>
-      <c r="E101" s="34"/>
-      <c r="F101" s="34"/>
-      <c r="G101" s="34"/>
-      <c r="H101" s="34"/>
-      <c r="I101" s="34"/>
-      <c r="J101" s="35"/>
+      <c r="C101" s="40"/>
+      <c r="D101" s="40"/>
+      <c r="E101" s="40"/>
+      <c r="F101" s="40"/>
+      <c r="G101" s="40"/>
+      <c r="H101" s="40"/>
+      <c r="I101" s="40"/>
+      <c r="J101" s="41"/>
     </row>
     <row r="102" spans="2:10" s="3" customFormat="1" ht="21" customHeight="1">
       <c r="B102" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="C102" s="34"/>
-      <c r="D102" s="34"/>
-      <c r="E102" s="34"/>
-      <c r="F102" s="34"/>
-      <c r="G102" s="34"/>
-      <c r="H102" s="34"/>
-      <c r="I102" s="34"/>
-      <c r="J102" s="35"/>
+      <c r="C102" s="40"/>
+      <c r="D102" s="40"/>
+      <c r="E102" s="40"/>
+      <c r="F102" s="40"/>
+      <c r="G102" s="40"/>
+      <c r="H102" s="40"/>
+      <c r="I102" s="40"/>
+      <c r="J102" s="41"/>
     </row>
     <row r="103" spans="2:10" ht="23.1" customHeight="1">
-      <c r="B103" s="52" t="s">
+      <c r="B103" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="C103" s="53"/>
-      <c r="D103" s="53"/>
-      <c r="E103" s="53"/>
-      <c r="F103" s="53"/>
-      <c r="G103" s="53"/>
-      <c r="H103" s="53"/>
-      <c r="I103" s="53"/>
-      <c r="J103" s="54"/>
+      <c r="C103" s="50"/>
+      <c r="D103" s="50"/>
+      <c r="E103" s="50"/>
+      <c r="F103" s="50"/>
+      <c r="G103" s="50"/>
+      <c r="H103" s="50"/>
+      <c r="I103" s="50"/>
+      <c r="J103" s="51"/>
     </row>
     <row r="104" spans="2:10" ht="23.1" customHeight="1">
-      <c r="B104" s="37"/>
-      <c r="C104" s="38"/>
-      <c r="D104" s="38"/>
-      <c r="E104" s="38"/>
-      <c r="F104" s="38"/>
-      <c r="G104" s="38"/>
-      <c r="H104" s="38"/>
-      <c r="I104" s="38"/>
-      <c r="J104" s="39"/>
+      <c r="B104" s="100"/>
+      <c r="C104" s="101"/>
+      <c r="D104" s="101"/>
+      <c r="E104" s="101"/>
+      <c r="F104" s="101"/>
+      <c r="G104" s="101"/>
+      <c r="H104" s="101"/>
+      <c r="I104" s="101"/>
+      <c r="J104" s="102"/>
     </row>
     <row r="105" spans="2:10" ht="23.1" customHeight="1">
-      <c r="B105" s="40"/>
-      <c r="C105" s="41"/>
-      <c r="D105" s="41"/>
-      <c r="E105" s="41"/>
-      <c r="F105" s="41"/>
-      <c r="G105" s="41"/>
-      <c r="H105" s="41"/>
-      <c r="I105" s="41"/>
-      <c r="J105" s="42"/>
+      <c r="B105" s="103"/>
+      <c r="C105" s="104"/>
+      <c r="D105" s="104"/>
+      <c r="E105" s="104"/>
+      <c r="F105" s="104"/>
+      <c r="G105" s="104"/>
+      <c r="H105" s="104"/>
+      <c r="I105" s="104"/>
+      <c r="J105" s="105"/>
     </row>
     <row r="106" spans="2:10" ht="23.1" customHeight="1">
-      <c r="B106" s="43"/>
-      <c r="C106" s="44"/>
-      <c r="D106" s="44"/>
-      <c r="E106" s="44"/>
-      <c r="F106" s="44"/>
-      <c r="G106" s="44"/>
-      <c r="H106" s="44"/>
-      <c r="I106" s="44"/>
-      <c r="J106" s="45"/>
-    </row>
-    <row r="107" spans="2:10" ht="18.75" customHeight="1">
-      <c r="B107" s="25" t="s">
+      <c r="B106" s="106"/>
+      <c r="C106" s="107"/>
+      <c r="D106" s="107"/>
+      <c r="E106" s="107"/>
+      <c r="F106" s="107"/>
+      <c r="G106" s="107"/>
+      <c r="H106" s="107"/>
+      <c r="I106" s="107"/>
+      <c r="J106" s="108"/>
+    </row>
+    <row r="107" spans="2:10" ht="228" customHeight="1">
+      <c r="B107" s="9"/>
+      <c r="C107" s="9"/>
+      <c r="D107" s="39"/>
+      <c r="E107" s="39"/>
+      <c r="F107" s="39"/>
+      <c r="G107" s="39"/>
+      <c r="H107" s="39"/>
+      <c r="I107" s="39"/>
+      <c r="J107" s="39"/>
+    </row>
+    <row r="108" spans="2:10" ht="62.4" customHeight="1">
+      <c r="B108" s="109"/>
+      <c r="C108" s="109"/>
+      <c r="D108" s="110"/>
+      <c r="E108" s="111"/>
+      <c r="F108" s="111"/>
+      <c r="G108" s="111"/>
+      <c r="H108" s="112"/>
+      <c r="I108" s="110"/>
+      <c r="J108" s="112"/>
+    </row>
+    <row r="109" spans="2:10" ht="18.75" customHeight="1">
+      <c r="B109" s="25" t="s">
         <v>115</v>
       </c>
-      <c r="C107" s="26"/>
-      <c r="D107" s="27"/>
-      <c r="E107" s="59" t="s">
+      <c r="C109" s="26"/>
+      <c r="D109" s="27"/>
+      <c r="E109" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="F107" s="59"/>
-      <c r="G107" s="59"/>
-      <c r="H107" s="59"/>
-      <c r="I107" s="59"/>
-      <c r="J107" s="60"/>
-    </row>
-    <row r="108" spans="2:10" ht="18.75" customHeight="1">
-      <c r="B108" s="28"/>
-      <c r="C108" s="29"/>
-      <c r="D108" s="30"/>
-      <c r="E108" s="61"/>
-      <c r="F108" s="61"/>
-      <c r="G108" s="61"/>
-      <c r="H108" s="61"/>
-      <c r="I108" s="61"/>
-      <c r="J108" s="62"/>
-    </row>
-    <row r="109" spans="2:10" ht="80.400000000000006" customHeight="1">
-      <c r="B109" s="31"/>
-      <c r="C109" s="32"/>
-      <c r="D109" s="33"/>
-      <c r="E109" s="63"/>
-      <c r="F109" s="63"/>
-      <c r="G109" s="63"/>
-      <c r="H109" s="63"/>
-      <c r="I109" s="63"/>
-      <c r="J109" s="64"/>
-    </row>
-    <row r="110" spans="2:10">
-      <c r="B110" s="3"/>
-      <c r="C110" s="3"/>
-      <c r="D110" s="3"/>
-      <c r="E110" s="3"/>
-      <c r="F110" s="3"/>
-      <c r="G110" s="3"/>
-      <c r="H110" s="3"/>
-      <c r="I110" s="3"/>
-      <c r="J110" s="3"/>
-    </row>
-    <row r="111" spans="2:10">
-      <c r="B111" s="3"/>
-      <c r="C111" s="3"/>
-      <c r="D111" s="3"/>
-      <c r="E111" s="3"/>
-      <c r="F111" s="3"/>
-      <c r="G111" s="3"/>
-      <c r="H111" s="3"/>
-      <c r="I111" s="3"/>
-      <c r="J111" s="3"/>
+      <c r="F109" s="58"/>
+      <c r="G109" s="58"/>
+      <c r="H109" s="58"/>
+      <c r="I109" s="58"/>
+      <c r="J109" s="59"/>
+    </row>
+    <row r="110" spans="2:10" ht="18.75" customHeight="1">
+      <c r="B110" s="28"/>
+      <c r="C110" s="29"/>
+      <c r="D110" s="30"/>
+      <c r="E110" s="60"/>
+      <c r="F110" s="60"/>
+      <c r="G110" s="60"/>
+      <c r="H110" s="60"/>
+      <c r="I110" s="60"/>
+      <c r="J110" s="61"/>
+    </row>
+    <row r="111" spans="2:10" ht="80.400000000000006" customHeight="1">
+      <c r="B111" s="31"/>
+      <c r="C111" s="32"/>
+      <c r="D111" s="33"/>
+      <c r="E111" s="62"/>
+      <c r="F111" s="62"/>
+      <c r="G111" s="62"/>
+      <c r="H111" s="62"/>
+      <c r="I111" s="62"/>
+      <c r="J111" s="63"/>
     </row>
     <row r="112" spans="2:10">
       <c r="B112" s="3"/>
@@ -3858,7 +3878,7 @@
       <c r="I112" s="3"/>
       <c r="J112" s="3"/>
     </row>
-    <row r="113" spans="2:9">
+    <row r="113" spans="2:10">
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
@@ -3867,8 +3887,9 @@
       <c r="G113" s="3"/>
       <c r="H113" s="3"/>
       <c r="I113" s="3"/>
-    </row>
-    <row r="114" spans="2:9">
+      <c r="J113" s="3"/>
+    </row>
+    <row r="114" spans="2:10">
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
       <c r="D114" s="3"/>
@@ -3877,8 +3898,9 @@
       <c r="G114" s="3"/>
       <c r="H114" s="3"/>
       <c r="I114" s="3"/>
-    </row>
-    <row r="115" spans="2:9">
+      <c r="J114" s="3"/>
+    </row>
+    <row r="115" spans="2:10">
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
       <c r="D115" s="3"/>
@@ -3888,7 +3910,7 @@
       <c r="H115" s="3"/>
       <c r="I115" s="3"/>
     </row>
-    <row r="116" spans="2:9">
+    <row r="116" spans="2:10">
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
       <c r="D116" s="3"/>
@@ -3898,7 +3920,7 @@
       <c r="H116" s="3"/>
       <c r="I116" s="3"/>
     </row>
-    <row r="117" spans="2:9">
+    <row r="117" spans="2:10">
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
       <c r="D117" s="3"/>
@@ -3908,7 +3930,7 @@
       <c r="H117" s="3"/>
       <c r="I117" s="3"/>
     </row>
-    <row r="118" spans="2:9">
+    <row r="118" spans="2:10">
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
@@ -3918,10 +3940,33 @@
       <c r="H118" s="3"/>
       <c r="I118" s="3"/>
     </row>
+    <row r="119" spans="2:10">
+      <c r="B119" s="3"/>
+      <c r="C119" s="3"/>
+      <c r="D119" s="3"/>
+      <c r="E119" s="3"/>
+      <c r="F119" s="3"/>
+      <c r="G119" s="3"/>
+      <c r="H119" s="3"/>
+      <c r="I119" s="3"/>
+    </row>
+    <row r="120" spans="2:10">
+      <c r="B120" s="3"/>
+      <c r="C120" s="3"/>
+      <c r="D120" s="3"/>
+      <c r="E120" s="3"/>
+      <c r="F120" s="3"/>
+      <c r="G120" s="3"/>
+      <c r="H120" s="3"/>
+      <c r="I120" s="3"/>
+    </row>
   </sheetData>
-  <mergeCells count="183">
-    <mergeCell ref="C100:E100"/>
-    <mergeCell ref="F93:H93"/>
+  <mergeCells count="187">
+    <mergeCell ref="C93:E93"/>
+    <mergeCell ref="C94:E94"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="C97:E97"/>
     <mergeCell ref="F94:H94"/>
     <mergeCell ref="F95:H95"/>
     <mergeCell ref="F96:H96"/>
@@ -3935,11 +3980,6 @@
     <mergeCell ref="I97:J97"/>
     <mergeCell ref="I98:J98"/>
     <mergeCell ref="I99:J99"/>
-    <mergeCell ref="C93:E93"/>
-    <mergeCell ref="C94:E94"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="C96:E96"/>
-    <mergeCell ref="C97:E97"/>
     <mergeCell ref="D7:G7"/>
     <mergeCell ref="D8:G8"/>
     <mergeCell ref="B27:C27"/>
@@ -4012,10 +4052,11 @@
     <mergeCell ref="B63:C63"/>
     <mergeCell ref="B65:C65"/>
     <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B64:C64"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="I36:J36"/>
     <mergeCell ref="C89:E89"/>
-    <mergeCell ref="E107:J109"/>
+    <mergeCell ref="E109:J111"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B73:C73"/>
     <mergeCell ref="B74:C74"/>
@@ -4036,8 +4077,6 @@
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="F89:H89"/>
     <mergeCell ref="F91:H91"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="I64:J64"/>
     <mergeCell ref="I85:J85"/>
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="F92:H92"/>
@@ -4060,6 +4099,8 @@
     <mergeCell ref="C101:J101"/>
     <mergeCell ref="C102:J102"/>
     <mergeCell ref="I91:J91"/>
+    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="F93:H93"/>
     <mergeCell ref="I42:J42"/>
     <mergeCell ref="I53:J53"/>
     <mergeCell ref="I54:J54"/>
@@ -4084,6 +4125,10 @@
     <mergeCell ref="I43:J43"/>
     <mergeCell ref="I44:J44"/>
     <mergeCell ref="I45:J45"/>
+    <mergeCell ref="D107:H107"/>
+    <mergeCell ref="I107:J107"/>
+    <mergeCell ref="D108:H108"/>
+    <mergeCell ref="I108:J108"/>
     <mergeCell ref="I47:J47"/>
     <mergeCell ref="I48:J48"/>
     <mergeCell ref="I50:J50"/>
@@ -4103,6 +4148,7 @@
     <mergeCell ref="I65:J65"/>
     <mergeCell ref="I66:J66"/>
     <mergeCell ref="I74:J74"/>
+    <mergeCell ref="I64:J64"/>
   </mergeCells>
   <phoneticPr fontId="22" type="noConversion"/>
   <dataValidations count="1">

</xml_diff>